<commit_message>
frontend/made some map changes
</commit_message>
<xml_diff>
--- a/backend/dependency_table_repo.xlsx
+++ b/backend/dependency_table_repo.xlsx
@@ -448,42 +448,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>347</t>
+          <t>1023</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Controller.php</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>348, 349, 350, 351, 352, 353</t>
-        </is>
-      </c>
+          <t>AuthController.php</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>348</t>
+          <t>1024</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CreateCapsuleController.php</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>Controller.php</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1025, 1026, 1027, 1028</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>349</t>
+          <t>1025</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DashboardController.php</t>
+          <t>CapsuleController.php</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -491,12 +491,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>1026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ProfileController.php</t>
+          <t>EmailController.php</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -504,12 +504,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>351</t>
+          <t>1027</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PublicWallController.php</t>
+          <t>MediaController.php</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -517,12 +517,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>1028</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ViewCapsuleController.php</t>
+          <t>UserController.php</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -530,115 +530,115 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>353</t>
+          <t>1030</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AuthController.php</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>Capsule.php</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1025, 1036, 1037</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>1031</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Capsule.php</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>349, 351, 352, 358, 359</t>
-        </is>
-      </c>
+          <t>Email.php</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>1032</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>User.php</t>
+          <t>Media.php</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>350, 351, 360, 361</t>
+          <t>1027, 1037</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>1033</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CapsuleRevealService.php</t>
+          <t>User.php</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>349, 351</t>
+          <t>1035</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>1035</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CapsuleService.php</t>
+          <t>AuthService.php</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>348</t>
+          <t>1023</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>1036</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>UserService.php</t>
+          <t>CapsuleService.php</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>1025</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>1037</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AuthService.php</t>
+          <t>MediaService.php</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>353</t>
+          <t>1027</t>
         </is>
       </c>
     </row>

</xml_diff>